<commit_message>
chore: weekly briefing 2026-10-09 23:00Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-10-06.xlsx
+++ b/public/reports/weekly_briefing/2026-10-06.xlsx
@@ -1014,7 +1014,7 @@
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>미국 종가 기준 10/05 → 10/07, %</t>
+          <t>미국 종가 기준 10/05 → 10/09, %</t>
         </is>
       </c>
       <c r="I6" s="18" t="inlineStr"/>
@@ -1084,19 +1084,19 @@
         <v>-23409</v>
       </c>
       <c r="E8" s="28" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="F8" s="29" t="n">
-        <v>-0.17</v>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>0.22</v>
+        <v>0.48</v>
+      </c>
+      <c r="F8" s="28" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G8" s="29" t="n">
+        <v>-0.4</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>-2.84</v>
+        <v>-4.38</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-4.56</v>
       </c>
     </row>
     <row r="9">
@@ -1151,11 +1151,11 @@
       </c>
       <c r="C12" s="31" t="inlineStr">
         <is>
-          <t>헬스케어</t>
+          <t>에너지</t>
         </is>
       </c>
       <c r="D12" s="32" t="n">
-        <v>0.86</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="13">
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="D13" s="32" t="n">
-        <v>0.85</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="14">
@@ -1191,11 +1191,11 @@
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>기술</t>
+          <t>헬스케어</t>
         </is>
       </c>
       <c r="D14" s="32" t="n">
-        <v>0.23</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="15">
@@ -1211,11 +1211,11 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
-          <t>바이오</t>
+          <t>반도체</t>
         </is>
       </c>
       <c r="D15" s="33" t="n">
-        <v>-3.82</v>
+        <v>-4.82</v>
       </c>
     </row>
     <row r="16">
@@ -1231,11 +1231,11 @@
       </c>
       <c r="C16" s="31" t="inlineStr">
         <is>
-          <t>반도체</t>
+          <t>바이오</t>
         </is>
       </c>
       <c r="D16" s="33" t="n">
-        <v>-1.4</v>
+        <v>-1.55</v>
       </c>
     </row>
     <row r="17">
@@ -1251,11 +1251,11 @@
       </c>
       <c r="C17" s="31" t="inlineStr">
         <is>
-          <t>산업재</t>
+          <t>기술</t>
         </is>
       </c>
       <c r="D17" s="33" t="n">
-        <v>-1.33</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="18">
@@ -11568,7 +11568,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{80519698-ADDF-4CFD-B553-314C4B2DA2C7}</x14:id>
+          <x14:id>{72FDA053-7919-440E-9D41-BCF7CCA83868}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11582,7 +11582,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A224DFAB-70A8-4BCE-BC40-E7BCC0567659}</x14:id>
+          <x14:id>{08507B12-1AB2-4EFD-8571-A18CE9E43C56}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11596,7 +11596,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F49D2038-F3D2-4417-9976-CD59C529557C}</x14:id>
+          <x14:id>{29597CC7-8A6F-4A32-9F06-1CCAA0992C59}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11610,7 +11610,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CD15E5B1-C234-4A12-9577-83D03ECFB78C}</x14:id>
+          <x14:id>{F9ED8B85-465F-4293-B292-3C7245EBB48B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -11620,7 +11620,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{80519698-ADDF-4CFD-B553-314C4B2DA2C7}">
+          <x14:cfRule type="dataBar" id="{72FDA053-7919-440E-9D41-BCF7CCA83868}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11633,7 +11633,7 @@
           <xm:sqref>B5:B28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A224DFAB-70A8-4BCE-BC40-E7BCC0567659}">
+          <x14:cfRule type="dataBar" id="{08507B12-1AB2-4EFD-8571-A18CE9E43C56}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11646,7 +11646,7 @@
           <xm:sqref>C5:C28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F49D2038-F3D2-4417-9976-CD59C529557C}">
+          <x14:cfRule type="dataBar" id="{29597CC7-8A6F-4A32-9F06-1CCAA0992C59}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -11659,7 +11659,7 @@
           <xm:sqref>D5:D28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CD15E5B1-C234-4A12-9577-83D03ECFB78C}">
+          <x14:cfRule type="dataBar" id="{F9ED8B85-465F-4293-B292-3C7245EBB48B}">
             <x14:dataBar minLength="0" maxLength="100" border="1" axisPosition="automatic" negativeBarColorSameAsPositive="0" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>